<commit_message>
graficos tema 4, Variabilidad y forma
</commit_message>
<xml_diff>
--- a/Ejemplos_Excel/Datos_Ejemplos.xlsx
+++ b/Ejemplos_Excel/Datos_Ejemplos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\Semestre 1-2026\Trabajo Dirigido\Proyecto\Proyecto_SHC170\Ejemplos_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007A9A2E-A25B-416D-84C4-40B44BE64870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8F2A77-BD02-49E7-A294-176B358D581A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" firstSheet="3" activeTab="6" xr2:uid="{F673EB76-743D-4B0D-96C3-C32891F51760}"/>
+    <workbookView xWindow="1620" yWindow="1590" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="7" xr2:uid="{F673EB76-743D-4B0D-96C3-C32891F51760}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Ej1" sheetId="2" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Intervalos_Ej2.5" sheetId="5" r:id="rId5"/>
     <sheet name="Ejemplo 2.9 (Bivariante)" sheetId="6" r:id="rId6"/>
     <sheet name="Ejemplo 4.10 (Pearson)" sheetId="7" r:id="rId7"/>
+    <sheet name="Ejemplo 3.57 (Box-Plot)" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="137">
   <si>
     <t>Datos 1</t>
   </si>
@@ -448,13 +449,16 @@
   </si>
   <si>
     <t>260.83</t>
+  </si>
+  <si>
+    <t>40 ejecutivos de marketing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -466,6 +470,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2411,4 +2421,223 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89DA3CF2-E51D-480C-92D7-6F2DE36953E8}">
+  <dimension ref="A1:A41"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
tema 6 y 7
</commit_message>
<xml_diff>
--- a/Ejemplos_Excel/Datos_Ejemplos.xlsx
+++ b/Ejemplos_Excel/Datos_Ejemplos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\Semestre 1-2026\Trabajo Dirigido\Proyecto\Proyecto_SHC170\Ejemplos_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8F2A77-BD02-49E7-A294-176B358D581A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B91487FC-AFAA-4F5C-BC87-CD0A7381EDF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="1590" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="7" xr2:uid="{F673EB76-743D-4B0D-96C3-C32891F51760}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="10" xr2:uid="{F673EB76-743D-4B0D-96C3-C32891F51760}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Ej1" sheetId="2" r:id="rId1"/>
@@ -21,6 +21,9 @@
     <sheet name="Ejemplo 2.9 (Bivariante)" sheetId="6" r:id="rId6"/>
     <sheet name="Ejemplo 4.10 (Pearson)" sheetId="7" r:id="rId7"/>
     <sheet name="Ejemplo 3.57 (Box-Plot)" sheetId="8" r:id="rId8"/>
+    <sheet name="Ejemplo 5.1" sheetId="9" r:id="rId9"/>
+    <sheet name="Ejemplo 5.6" sheetId="10" r:id="rId10"/>
+    <sheet name="Hoja3" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="148">
   <si>
     <t>Datos 1</t>
   </si>
@@ -452,6 +455,39 @@
   </si>
   <si>
     <t>40 ejecutivos de marketing</t>
+  </si>
+  <si>
+    <t>Periodo</t>
+  </si>
+  <si>
+    <t>3.7</t>
+  </si>
+  <si>
+    <t>21.6</t>
+  </si>
+  <si>
+    <t>37.6</t>
+  </si>
+  <si>
+    <t>6.1</t>
+  </si>
+  <si>
+    <t>Total ventas (Y)</t>
+  </si>
+  <si>
+    <t>Publicidad (X)</t>
+  </si>
+  <si>
+    <t>Gastos en alimentacion</t>
+  </si>
+  <si>
+    <t>Ingreso</t>
+  </si>
+  <si>
+    <t>Horas</t>
+  </si>
+  <si>
+    <t>Satisfacción en el trabajo</t>
   </si>
 </sst>
 </file>
@@ -501,7 +537,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -521,6 +557,18 @@
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -900,6 +948,481 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C53ABA-7916-4CB1-8FED-A33FDB0CD5F9}">
+  <dimension ref="A1:B35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.28515625" style="8" customWidth="1"/>
+    <col min="2" max="16384" width="11.42578125" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>2000</v>
+      </c>
+      <c r="B2" s="8">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>1500</v>
+      </c>
+      <c r="B3" s="8">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>3000</v>
+      </c>
+      <c r="B4" s="8">
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>4500</v>
+      </c>
+      <c r="B5" s="8">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>6000</v>
+      </c>
+      <c r="B6" s="8">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>6500</v>
+      </c>
+      <c r="B7" s="8">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>1500</v>
+      </c>
+      <c r="B8" s="8">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>1500</v>
+      </c>
+      <c r="B9" s="8">
+        <v>5550</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>1580</v>
+      </c>
+      <c r="B10" s="8">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>2500</v>
+      </c>
+      <c r="B11" s="8">
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>2500</v>
+      </c>
+      <c r="B12" s="8">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>4000</v>
+      </c>
+      <c r="B13" s="8">
+        <v>5600</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="8">
+        <v>5600</v>
+      </c>
+      <c r="B14" s="8">
+        <v>10200</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>5300</v>
+      </c>
+      <c r="B15" s="8">
+        <v>8500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="8">
+        <v>4600</v>
+      </c>
+      <c r="B16" s="8">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="8">
+        <v>4500</v>
+      </c>
+      <c r="B17" s="8">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="8">
+        <v>3500</v>
+      </c>
+      <c r="B18" s="8">
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="8">
+        <v>2800</v>
+      </c>
+      <c r="B19" s="8">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="8">
+        <v>3020</v>
+      </c>
+      <c r="B20" s="8">
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="8">
+        <v>2500</v>
+      </c>
+      <c r="B21" s="8">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="8">
+        <v>5600</v>
+      </c>
+      <c r="B22" s="8">
+        <v>11500</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="8">
+        <v>8000</v>
+      </c>
+      <c r="B23" s="8">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="8">
+        <v>10000</v>
+      </c>
+      <c r="B24" s="8">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="8">
+        <v>6500</v>
+      </c>
+      <c r="B25" s="8">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="8">
+        <v>4500</v>
+      </c>
+      <c r="B26" s="8">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="8">
+        <v>6000</v>
+      </c>
+      <c r="B27" s="8">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="8">
+        <v>5300</v>
+      </c>
+      <c r="B28" s="8">
+        <v>10500</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="8">
+        <v>7500</v>
+      </c>
+      <c r="B29" s="8">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="8">
+        <v>2300</v>
+      </c>
+      <c r="B30" s="8">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="8">
+        <v>2800</v>
+      </c>
+      <c r="B31" s="8">
+        <v>5600</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="8">
+        <v>7500</v>
+      </c>
+      <c r="B32" s="8">
+        <v>15500</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="8">
+        <v>2000</v>
+      </c>
+      <c r="B33" s="8">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="8">
+        <v>6500</v>
+      </c>
+      <c r="B34" s="8">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="8">
+        <v>6500</v>
+      </c>
+      <c r="B35" s="8">
+        <v>17000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{066FAF81-566D-484C-83F8-1E7D9A3EBB16}">
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="11.42578125" style="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="11">
+        <v>70</v>
+      </c>
+      <c r="B2" s="11">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="11">
+        <v>80</v>
+      </c>
+      <c r="B3" s="11">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="11">
+        <v>80</v>
+      </c>
+      <c r="B4" s="11">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="11">
+        <v>70</v>
+      </c>
+      <c r="B5" s="11">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="11">
+        <v>85</v>
+      </c>
+      <c r="B6" s="11">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="11">
+        <v>70</v>
+      </c>
+      <c r="B7" s="11">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="11">
+        <v>35</v>
+      </c>
+      <c r="B8" s="11">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="11">
+        <v>90</v>
+      </c>
+      <c r="B9" s="11">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="11">
+        <v>85</v>
+      </c>
+      <c r="B10" s="11">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="11">
+        <v>65</v>
+      </c>
+      <c r="B11" s="11">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="11">
+        <v>85</v>
+      </c>
+      <c r="B12" s="11">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="11">
+        <v>75</v>
+      </c>
+      <c r="B13" s="11">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="11">
+        <v>75</v>
+      </c>
+      <c r="B14" s="11">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="11">
+        <v>80</v>
+      </c>
+      <c r="B15" s="11">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="11">
+        <v>50</v>
+      </c>
+      <c r="B16" s="11">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="11">
+        <v>70</v>
+      </c>
+      <c r="B17" s="11">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="11">
+        <v>80</v>
+      </c>
+      <c r="B18" s="11">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="11">
+        <v>60</v>
+      </c>
+      <c r="B19" s="11">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="11">
+        <v>65</v>
+      </c>
+      <c r="B20" s="11">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="11">
+        <v>30</v>
+      </c>
+      <c r="B21" s="11">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5286FA33-8335-4F16-8FFE-4911A034FBC6}">
   <dimension ref="A1:B7"/>
@@ -2640,4 +3163,141 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8381F06-0351-45EA-8205-A1AB884EB138}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.5703125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" style="8" customWidth="1"/>
+    <col min="4" max="16384" width="11.42578125" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8">
+        <v>150</v>
+      </c>
+      <c r="C2" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8">
+        <v>75</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8">
+        <v>338</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8">
+        <v>750</v>
+      </c>
+      <c r="C5" s="8">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8">
+        <v>541</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8">
+        <v>89</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8">
+        <v>126</v>
+      </c>
+      <c r="C8" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8">
+        <v>379</v>
+      </c>
+      <c r="C9" s="8">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8">
+        <v>650</v>
+      </c>
+      <c r="C10" s="8">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8">
+        <v>350</v>
+      </c>
+      <c r="C11" s="8">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: eliminar seleccion por fila e integrar banner de entorno beta
</commit_message>
<xml_diff>
--- a/Ejemplos_Excel/Datos_Ejemplos.xlsx
+++ b/Ejemplos_Excel/Datos_Ejemplos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\Semestre 1-2026\Trabajo Dirigido\Proyecto\Proyecto_SHC170\Ejemplos_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC398FAD-0C45-4E61-B2E5-B693ABD3FD55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07253135-AF36-4B9C-A259-4E30D9FDD038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11130" yWindow="2370" windowWidth="14730" windowHeight="11295" firstSheet="11" activeTab="13" xr2:uid="{F673EB76-743D-4B0D-96C3-C32891F51760}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" firstSheet="11" activeTab="12" xr2:uid="{F673EB76-743D-4B0D-96C3-C32891F51760}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Ej1" sheetId="2" r:id="rId1"/>
@@ -25,8 +25,9 @@
     <sheet name="Ejemplo 5.8 (Regresion)" sheetId="11" r:id="rId10"/>
     <sheet name="Ejemplo 6.1 (N.Indices)" sheetId="14" r:id="rId11"/>
     <sheet name="Ejemplo 6.2 (N.Indices)" sheetId="15" r:id="rId12"/>
-    <sheet name="Ejemplo 5.7 (Regresion Cuad.)" sheetId="16" r:id="rId13"/>
-    <sheet name="Ejemplo 6.9 (N. Indice)" sheetId="17" r:id="rId14"/>
+    <sheet name="Hoja1" sheetId="18" r:id="rId13"/>
+    <sheet name="Ejemplo 5.7 (Regresion Cuad.)" sheetId="16" r:id="rId14"/>
+    <sheet name="Ejemplo 6.9 (N. Indice)" sheetId="17" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1709,6 +1710,98 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77BD8D67-1733-43C7-B549-946A534FFF6F}">
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>2</v>
+      </c>
+      <c r="B1">
+        <v>5</v>
+      </c>
+      <c r="C1">
+        <v>6</v>
+      </c>
+      <c r="D1">
+        <v>10</v>
+      </c>
+      <c r="E1">
+        <v>85</v>
+      </c>
+      <c r="F1">
+        <v>10</v>
+      </c>
+      <c r="G1">
+        <v>58</v>
+      </c>
+      <c r="H1">
+        <v>45</v>
+      </c>
+      <c r="I1">
+        <v>5</v>
+      </c>
+      <c r="J1">
+        <v>6</v>
+      </c>
+      <c r="K1">
+        <v>7</v>
+      </c>
+      <c r="L1">
+        <v>8</v>
+      </c>
+      <c r="M1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>6</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>8</v>
+      </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+      <c r="M2">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68B0B285-2017-4174-A96C-88E1B3B82AD1}">
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1809,7 +1902,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F000942-8A84-46B3-8480-9C5561E0F5A1}">
   <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>